<commit_message>
feat: refresh store furniture artwork and per-item footprints
</commit_message>
<xml_diff>
--- a/Excel/家具表.xlsx
+++ b/Excel/家具表.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="家具" sheetId="1" r:id="R41c6267c0f8a4dff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="家具" sheetId="1" r:id="R3c458a2154e54295"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -346,6 +346,10 @@
     <x:col min="8" max="8" width="10" customWidth="1"/>
     <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="50" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="50" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="10" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="10" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -395,6 +399,18 @@
       <x:c r="J1" t="str">
         <x:v>商店显示高</x:v>
       </x:c>
+      <x:c r="K1" t="str">
+        <x:v>商店列表图</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>商店详情图</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>占格列</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>占格行</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="1" t="inlineStr">
@@ -443,6 +459,18 @@
       <x:c r="J2" t="str">
         <x:v>storeDisplayHeight</x:v>
       </x:c>
+      <x:c r="K2" t="str">
+        <x:v>storeListSprite</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>storePreviewSprite</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>cols</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>rows</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="inlineStr">
@@ -485,6 +513,18 @@
       <x:c r="J3" t="n">
         <x:v>220</x:v>
       </x:c>
+      <x:c r="K3" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/台灯-1.png</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/台灯-1.png</x:v>
+      </x:c>
+      <x:c r="M3" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N3" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="inlineStr">
@@ -527,6 +567,18 @@
       <x:c r="J4" t="n">
         <x:v>220</x:v>
       </x:c>
+      <x:c r="K4" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/台灯-2.png</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/台灯-2.png</x:v>
+      </x:c>
+      <x:c r="M4" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N4" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="inlineStr">
@@ -569,6 +621,18 @@
       <x:c r="J5" t="n">
         <x:v>220</x:v>
       </x:c>
+      <x:c r="K5" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/台灯-3.png</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/台灯-3.png</x:v>
+      </x:c>
+      <x:c r="M5" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N5" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="inlineStr">
@@ -611,6 +675,18 @@
       <x:c r="J6" t="n">
         <x:v>220</x:v>
       </x:c>
+      <x:c r="K6" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/台灯-4.png</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/台灯-4.png</x:v>
+      </x:c>
+      <x:c r="M6" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N6" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="inlineStr">
@@ -653,6 +729,18 @@
       <x:c r="J7" t="n">
         <x:v>220</x:v>
       </x:c>
+      <x:c r="K7" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/台灯-5.png</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/台灯-5.png</x:v>
+      </x:c>
+      <x:c r="M7" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N7" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="inlineStr">
@@ -695,6 +783,18 @@
       <x:c r="J8" t="n">
         <x:v>220</x:v>
       </x:c>
+      <x:c r="K8" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/台灯-6.png</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/台灯-6.png</x:v>
+      </x:c>
+      <x:c r="M8" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N8" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="inlineStr">
@@ -737,6 +837,14 @@
       <x:c r="J9" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K9" t="str"/>
+      <x:c r="L9" t="str"/>
+      <x:c r="M9" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N9" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="inlineStr">
@@ -779,6 +887,14 @@
       <x:c r="J10" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K10" t="str"/>
+      <x:c r="L10" t="str"/>
+      <x:c r="M10" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N10" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="inlineStr">
@@ -821,6 +937,14 @@
       <x:c r="J11" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K11" t="str"/>
+      <x:c r="L11" t="str"/>
+      <x:c r="M11" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N11" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="inlineStr">
@@ -863,6 +987,14 @@
       <x:c r="J12" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K12" t="str"/>
+      <x:c r="L12" t="str"/>
+      <x:c r="M12" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N12" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="inlineStr">
@@ -905,6 +1037,14 @@
       <x:c r="J13" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K13" t="str"/>
+      <x:c r="L13" t="str"/>
+      <x:c r="M13" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N13" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="inlineStr">
@@ -947,6 +1087,14 @@
       <x:c r="J14" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K14" t="str"/>
+      <x:c r="L14" t="str"/>
+      <x:c r="M14" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N14" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="inlineStr">
@@ -989,6 +1137,14 @@
       <x:c r="J15" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K15" t="str"/>
+      <x:c r="L15" t="str"/>
+      <x:c r="M15" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N15" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="inlineStr">
@@ -1031,6 +1187,14 @@
       <x:c r="J16" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K16" t="str"/>
+      <x:c r="L16" t="str"/>
+      <x:c r="M16" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N16" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="inlineStr">
@@ -1073,6 +1237,14 @@
       <x:c r="J17" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K17" t="str"/>
+      <x:c r="L17" t="str"/>
+      <x:c r="M17" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N17" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="inlineStr">
@@ -1115,6 +1287,14 @@
       <x:c r="J18" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K18" t="str"/>
+      <x:c r="L18" t="str"/>
+      <x:c r="M18" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N18" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="inlineStr">
@@ -1157,6 +1337,14 @@
       <x:c r="J19" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K19" t="str"/>
+      <x:c r="L19" t="str"/>
+      <x:c r="M19" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N19" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="inlineStr">
@@ -1199,6 +1387,14 @@
       <x:c r="J20" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K20" t="str"/>
+      <x:c r="L20" t="str"/>
+      <x:c r="M20" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N20" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="inlineStr">
@@ -1241,6 +1437,14 @@
       <x:c r="J21" t="n">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="K21" t="str"/>
+      <x:c r="L21" t="str"/>
+      <x:c r="M21" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N21" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="inlineStr">
@@ -1283,6 +1487,14 @@
       <x:c r="J22" t="n">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="K22" t="str"/>
+      <x:c r="L22" t="str"/>
+      <x:c r="M22" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N22" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="inlineStr">
@@ -1325,6 +1537,14 @@
       <x:c r="J23" t="n">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="K23" t="str"/>
+      <x:c r="L23" t="str"/>
+      <x:c r="M23" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N23" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="inlineStr">
@@ -1367,6 +1587,14 @@
       <x:c r="J24" t="n">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="K24" t="str"/>
+      <x:c r="L24" t="str"/>
+      <x:c r="M24" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N24" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="inlineStr">
@@ -1409,6 +1637,14 @@
       <x:c r="J25" t="n">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="K25" t="str"/>
+      <x:c r="L25" t="str"/>
+      <x:c r="M25" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N25" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="inlineStr">
@@ -1451,6 +1687,14 @@
       <x:c r="J26" t="n">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="K26" t="str"/>
+      <x:c r="L26" t="str"/>
+      <x:c r="M26" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N26" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="inlineStr">
@@ -1493,6 +1737,14 @@
       <x:c r="J27" t="n">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="K27" t="str"/>
+      <x:c r="L27" t="str"/>
+      <x:c r="M27" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N27" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="inlineStr">
@@ -1535,6 +1787,14 @@
       <x:c r="J28" t="n">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="K28" t="str"/>
+      <x:c r="L28" t="str"/>
+      <x:c r="M28" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N28" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="inlineStr">
@@ -1577,6 +1837,18 @@
       <x:c r="J29" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K29" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_10 3.png</x:v>
+      </x:c>
+      <x:c r="L29" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_10 2.png</x:v>
+      </x:c>
+      <x:c r="M29" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N29" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="inlineStr">
@@ -1619,6 +1891,18 @@
       <x:c r="J30" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K30" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_04 3.png</x:v>
+      </x:c>
+      <x:c r="L30" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_04 2.png</x:v>
+      </x:c>
+      <x:c r="M30" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N30" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="inlineStr">
@@ -1661,6 +1945,18 @@
       <x:c r="J31" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K31" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_09 3.png</x:v>
+      </x:c>
+      <x:c r="L31" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_09 2.png</x:v>
+      </x:c>
+      <x:c r="M31" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N31" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="inlineStr">
@@ -1703,6 +1999,18 @@
       <x:c r="J32" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K32" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_05 3.png</x:v>
+      </x:c>
+      <x:c r="L32" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_05 2.png</x:v>
+      </x:c>
+      <x:c r="M32" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N32" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="inlineStr">
@@ -1745,6 +2053,18 @@
       <x:c r="J33" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K33" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_06 3.png</x:v>
+      </x:c>
+      <x:c r="L33" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_06 2.png</x:v>
+      </x:c>
+      <x:c r="M33" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N33" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="inlineStr">
@@ -1787,6 +2107,18 @@
       <x:c r="J34" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K34" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_07 3.png</x:v>
+      </x:c>
+      <x:c r="L34" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_07 2.png</x:v>
+      </x:c>
+      <x:c r="M34" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N34" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="inlineStr">
@@ -1829,6 +2161,18 @@
       <x:c r="J35" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K35" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_08 3.png</x:v>
+      </x:c>
+      <x:c r="L35" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_08 2.png</x:v>
+      </x:c>
+      <x:c r="M35" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N35" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="inlineStr">
@@ -1871,6 +2215,18 @@
       <x:c r="J36" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K36" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_01 3.png</x:v>
+      </x:c>
+      <x:c r="L36" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_01 2.png</x:v>
+      </x:c>
+      <x:c r="M36" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N36" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="inlineStr">
@@ -1913,6 +2269,18 @@
       <x:c r="J37" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K37" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_02 3.png</x:v>
+      </x:c>
+      <x:c r="L37" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_02 2.png</x:v>
+      </x:c>
+      <x:c r="M37" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N37" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="inlineStr">
@@ -1955,6 +2323,18 @@
       <x:c r="J38" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K38" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_11 3.png</x:v>
+      </x:c>
+      <x:c r="L38" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_11 2.png</x:v>
+      </x:c>
+      <x:c r="M38" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N38" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" t="inlineStr">
@@ -1997,6 +2377,18 @@
       <x:c r="J39" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K39" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_12 3.png</x:v>
+      </x:c>
+      <x:c r="L39" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_12 2.png</x:v>
+      </x:c>
+      <x:c r="M39" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N39" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" t="inlineStr">
@@ -2039,6 +2431,18 @@
       <x:c r="J40" t="n">
         <x:v>160</x:v>
       </x:c>
+      <x:c r="K40" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/armchair_03 3.png</x:v>
+      </x:c>
+      <x:c r="L40" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/armchair_03 2.png</x:v>
+      </x:c>
+      <x:c r="M40" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N40" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" t="inlineStr">
@@ -2081,6 +2485,14 @@
       <x:c r="J41" t="n">
         <x:v>105</x:v>
       </x:c>
+      <x:c r="K41" t="str"/>
+      <x:c r="L41" t="str"/>
+      <x:c r="M41" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N41" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" t="inlineStr">
@@ -2123,6 +2535,14 @@
       <x:c r="J42" t="n">
         <x:v>105</x:v>
       </x:c>
+      <x:c r="K42" t="str"/>
+      <x:c r="L42" t="str"/>
+      <x:c r="M42" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N42" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" t="inlineStr">
@@ -2165,6 +2585,14 @@
       <x:c r="J43" t="n">
         <x:v>105</x:v>
       </x:c>
+      <x:c r="K43" t="str"/>
+      <x:c r="L43" t="str"/>
+      <x:c r="M43" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N43" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" t="inlineStr">
@@ -2207,6 +2635,14 @@
       <x:c r="J44" t="n">
         <x:v>105</x:v>
       </x:c>
+      <x:c r="K44" t="str"/>
+      <x:c r="L44" t="str"/>
+      <x:c r="M44" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N44" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" t="inlineStr">
@@ -2249,6 +2685,14 @@
       <x:c r="J45" t="n">
         <x:v>105</x:v>
       </x:c>
+      <x:c r="K45" t="str"/>
+      <x:c r="L45" t="str"/>
+      <x:c r="M45" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N45" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" t="inlineStr">
@@ -2291,6 +2735,14 @@
       <x:c r="J46" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K46" t="str"/>
+      <x:c r="L46" t="str"/>
+      <x:c r="M46" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N46" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" t="inlineStr">
@@ -2333,6 +2785,14 @@
       <x:c r="J47" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K47" t="str"/>
+      <x:c r="L47" t="str"/>
+      <x:c r="M47" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N47" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" t="inlineStr">
@@ -2375,6 +2835,14 @@
       <x:c r="J48" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K48" t="str"/>
+      <x:c r="L48" t="str"/>
+      <x:c r="M48" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N48" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" t="inlineStr">
@@ -2417,6 +2885,14 @@
       <x:c r="J49" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K49" t="str"/>
+      <x:c r="L49" t="str"/>
+      <x:c r="M49" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N49" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" t="inlineStr">
@@ -2459,6 +2935,14 @@
       <x:c r="J50" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K50" t="str"/>
+      <x:c r="L50" t="str"/>
+      <x:c r="M50" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N50" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" t="inlineStr">
@@ -2501,6 +2985,14 @@
       <x:c r="J51" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K51" t="str"/>
+      <x:c r="L51" t="str"/>
+      <x:c r="M51" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N51" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" t="inlineStr">
@@ -2543,6 +3035,14 @@
       <x:c r="J52" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K52" t="str"/>
+      <x:c r="L52" t="str"/>
+      <x:c r="M52" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N52" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" t="inlineStr">
@@ -2585,6 +3085,14 @@
       <x:c r="J53" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K53" t="str"/>
+      <x:c r="L53" t="str"/>
+      <x:c r="M53" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N53" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" t="inlineStr">
@@ -2627,6 +3135,14 @@
       <x:c r="J54" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K54" t="str"/>
+      <x:c r="L54" t="str"/>
+      <x:c r="M54" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N54" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" t="inlineStr">
@@ -2669,6 +3185,14 @@
       <x:c r="J55" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K55" t="str"/>
+      <x:c r="L55" t="str"/>
+      <x:c r="M55" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N55" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" t="inlineStr">
@@ -2711,6 +3235,14 @@
       <x:c r="J56" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K56" t="str"/>
+      <x:c r="L56" t="str"/>
+      <x:c r="M56" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N56" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" t="inlineStr">
@@ -2753,6 +3285,14 @@
       <x:c r="J57" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K57" t="str"/>
+      <x:c r="L57" t="str"/>
+      <x:c r="M57" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N57" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" t="inlineStr">
@@ -2795,6 +3335,14 @@
       <x:c r="J58" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K58" t="str"/>
+      <x:c r="L58" t="str"/>
+      <x:c r="M58" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N58" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" t="inlineStr">
@@ -2837,6 +3385,14 @@
       <x:c r="J59" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K59" t="str"/>
+      <x:c r="L59" t="str"/>
+      <x:c r="M59" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N59" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" t="inlineStr">
@@ -2879,6 +3435,14 @@
       <x:c r="J60" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K60" t="str"/>
+      <x:c r="L60" t="str"/>
+      <x:c r="M60" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N60" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" t="inlineStr">
@@ -2921,6 +3485,14 @@
       <x:c r="J61" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K61" t="str"/>
+      <x:c r="L61" t="str"/>
+      <x:c r="M61" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N61" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" t="inlineStr">
@@ -2963,6 +3535,14 @@
       <x:c r="J62" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K62" t="str"/>
+      <x:c r="L62" t="str"/>
+      <x:c r="M62" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N62" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" t="inlineStr">
@@ -3005,6 +3585,14 @@
       <x:c r="J63" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K63" t="str"/>
+      <x:c r="L63" t="str"/>
+      <x:c r="M63" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N63" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" t="inlineStr">
@@ -3047,6 +3635,14 @@
       <x:c r="J64" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K64" t="str"/>
+      <x:c r="L64" t="str"/>
+      <x:c r="M64" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N64" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" t="inlineStr">
@@ -3089,6 +3685,14 @@
       <x:c r="J65" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K65" t="str"/>
+      <x:c r="L65" t="str"/>
+      <x:c r="M65" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N65" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" t="inlineStr">
@@ -3131,6 +3735,14 @@
       <x:c r="J66" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K66" t="str"/>
+      <x:c r="L66" t="str"/>
+      <x:c r="M66" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N66" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" t="inlineStr">
@@ -3173,6 +3785,14 @@
       <x:c r="J67" t="n">
         <x:v>140</x:v>
       </x:c>
+      <x:c r="K67" t="str"/>
+      <x:c r="L67" t="str"/>
+      <x:c r="M67" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N67" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" t="inlineStr">
@@ -3215,6 +3835,14 @@
       <x:c r="J68" t="n">
         <x:v>135</x:v>
       </x:c>
+      <x:c r="K68" t="str"/>
+      <x:c r="L68" t="str"/>
+      <x:c r="M68" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N68" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" t="inlineStr">
@@ -3257,6 +3885,14 @@
       <x:c r="J69" t="n">
         <x:v>135</x:v>
       </x:c>
+      <x:c r="K69" t="str"/>
+      <x:c r="L69" t="str"/>
+      <x:c r="M69" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N69" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" t="inlineStr">
@@ -3299,6 +3935,14 @@
       <x:c r="J70" t="n">
         <x:v>135</x:v>
       </x:c>
+      <x:c r="K70" t="str"/>
+      <x:c r="L70" t="str"/>
+      <x:c r="M70" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N70" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" t="inlineStr">
@@ -3341,6 +3985,14 @@
       <x:c r="J71" t="n">
         <x:v>135</x:v>
       </x:c>
+      <x:c r="K71" t="str"/>
+      <x:c r="L71" t="str"/>
+      <x:c r="M71" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N71" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" t="inlineStr">
@@ -3383,6 +4035,14 @@
       <x:c r="J72" t="n">
         <x:v>135</x:v>
       </x:c>
+      <x:c r="K72" t="str"/>
+      <x:c r="L72" t="str"/>
+      <x:c r="M72" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N72" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" t="inlineStr">
@@ -3425,6 +4085,14 @@
       <x:c r="J73" t="n">
         <x:v>135</x:v>
       </x:c>
+      <x:c r="K73" t="str"/>
+      <x:c r="L73" t="str"/>
+      <x:c r="M73" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N73" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" t="inlineStr">
@@ -3467,6 +4135,14 @@
       <x:c r="J74" t="n">
         <x:v>135</x:v>
       </x:c>
+      <x:c r="K74" t="str"/>
+      <x:c r="L74" t="str"/>
+      <x:c r="M74" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N74" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" t="inlineStr">
@@ -3509,6 +4185,14 @@
       <x:c r="J75" t="n">
         <x:v>135</x:v>
       </x:c>
+      <x:c r="K75" t="str"/>
+      <x:c r="L75" t="str"/>
+      <x:c r="M75" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N75" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" t="inlineStr">
@@ -3551,6 +4235,18 @@
       <x:c r="J76" t="n">
         <x:v>125</x:v>
       </x:c>
+      <x:c r="K76" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/立式灯柱-1.png</x:v>
+      </x:c>
+      <x:c r="L76" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/立式灯柱-1.png</x:v>
+      </x:c>
+      <x:c r="M76" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N76" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" t="inlineStr">
@@ -3593,6 +4289,18 @@
       <x:c r="J77" t="n">
         <x:v>125</x:v>
       </x:c>
+      <x:c r="K77" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/立式灯柱-2.png</x:v>
+      </x:c>
+      <x:c r="L77" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/立式灯柱-2.png</x:v>
+      </x:c>
+      <x:c r="M77" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N77" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" t="inlineStr">
@@ -3635,6 +4343,18 @@
       <x:c r="J78" t="n">
         <x:v>125</x:v>
       </x:c>
+      <x:c r="K78" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/立式灯柱-3.png</x:v>
+      </x:c>
+      <x:c r="L78" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/立式灯柱-3.png</x:v>
+      </x:c>
+      <x:c r="M78" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N78" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="inlineStr">
@@ -3677,6 +4397,18 @@
       <x:c r="J79" t="n">
         <x:v>125</x:v>
       </x:c>
+      <x:c r="K79" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/立式灯柱-4.png</x:v>
+      </x:c>
+      <x:c r="L79" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/立式灯柱-4.png</x:v>
+      </x:c>
+      <x:c r="M79" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N79" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" t="inlineStr">
@@ -3719,6 +4451,18 @@
       <x:c r="J80" t="n">
         <x:v>125</x:v>
       </x:c>
+      <x:c r="K80" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/立式灯柱-5.png</x:v>
+      </x:c>
+      <x:c r="L80" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/立式灯柱-5.png</x:v>
+      </x:c>
+      <x:c r="M80" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N80" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" t="inlineStr">
@@ -3761,6 +4505,18 @@
       <x:c r="J81" t="n">
         <x:v>125</x:v>
       </x:c>
+      <x:c r="K81" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/立式灯柱-6.png</x:v>
+      </x:c>
+      <x:c r="L81" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/立式灯柱-6.png</x:v>
+      </x:c>
+      <x:c r="M81" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N81" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" t="inlineStr">
@@ -3803,6 +4559,18 @@
       <x:c r="J82" t="n">
         <x:v>125</x:v>
       </x:c>
+      <x:c r="K82" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/立式灯柱-7.png</x:v>
+      </x:c>
+      <x:c r="L82" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/立式灯柱-7.png</x:v>
+      </x:c>
+      <x:c r="M82" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N82" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" t="inlineStr">
@@ -3845,6 +4613,18 @@
       <x:c r="J83" t="n">
         <x:v>125</x:v>
       </x:c>
+      <x:c r="K83" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/立式灯柱-8.png</x:v>
+      </x:c>
+      <x:c r="L83" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/立式灯柱-8.png</x:v>
+      </x:c>
+      <x:c r="M83" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N83" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" t="inlineStr">
@@ -3887,6 +4667,14 @@
       <x:c r="J84" t="n">
         <x:v>205</x:v>
       </x:c>
+      <x:c r="K84" t="str"/>
+      <x:c r="L84" t="str"/>
+      <x:c r="M84" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N84" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" t="inlineStr">
@@ -3929,6 +4717,14 @@
       <x:c r="J85" t="n">
         <x:v>205</x:v>
       </x:c>
+      <x:c r="K85" t="str"/>
+      <x:c r="L85" t="str"/>
+      <x:c r="M85" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N85" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" t="inlineStr">
@@ -3971,6 +4767,14 @@
       <x:c r="J86" t="n">
         <x:v>205</x:v>
       </x:c>
+      <x:c r="K86" t="str"/>
+      <x:c r="L86" t="str"/>
+      <x:c r="M86" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N86" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" t="inlineStr">
@@ -4013,6 +4817,14 @@
       <x:c r="J87" t="n">
         <x:v>205</x:v>
       </x:c>
+      <x:c r="K87" t="str"/>
+      <x:c r="L87" t="str"/>
+      <x:c r="M87" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N87" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" t="inlineStr">
@@ -4055,6 +4867,14 @@
       <x:c r="J88" t="n">
         <x:v>205</x:v>
       </x:c>
+      <x:c r="K88" t="str"/>
+      <x:c r="L88" t="str"/>
+      <x:c r="M88" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N88" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" t="inlineStr">
@@ -4097,6 +4917,14 @@
       <x:c r="J89" t="n">
         <x:v>205</x:v>
       </x:c>
+      <x:c r="K89" t="str"/>
+      <x:c r="L89" t="str"/>
+      <x:c r="M89" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N89" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" t="inlineStr">
@@ -4139,6 +4967,14 @@
       <x:c r="J90" t="n">
         <x:v>205</x:v>
       </x:c>
+      <x:c r="K90" t="str"/>
+      <x:c r="L90" t="str"/>
+      <x:c r="M90" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N90" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" t="inlineStr">
@@ -4181,6 +5017,14 @@
       <x:c r="J91" t="n">
         <x:v>85</x:v>
       </x:c>
+      <x:c r="K91" t="str"/>
+      <x:c r="L91" t="str"/>
+      <x:c r="M91" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N91" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" t="inlineStr">
@@ -4223,6 +5067,14 @@
       <x:c r="J92" t="n">
         <x:v>85</x:v>
       </x:c>
+      <x:c r="K92" t="str"/>
+      <x:c r="L92" t="str"/>
+      <x:c r="M92" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N92" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" t="inlineStr">
@@ -4265,6 +5117,14 @@
       <x:c r="J93" t="n">
         <x:v>85</x:v>
       </x:c>
+      <x:c r="K93" t="str"/>
+      <x:c r="L93" t="str"/>
+      <x:c r="M93" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N93" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" t="inlineStr">
@@ -4307,6 +5167,14 @@
       <x:c r="J94" t="n">
         <x:v>85</x:v>
       </x:c>
+      <x:c r="K94" t="str"/>
+      <x:c r="L94" t="str"/>
+      <x:c r="M94" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N94" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" t="inlineStr">
@@ -4349,6 +5217,14 @@
       <x:c r="J95" t="n">
         <x:v>85</x:v>
       </x:c>
+      <x:c r="K95" t="str"/>
+      <x:c r="L95" t="str"/>
+      <x:c r="M95" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N95" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="96">
       <x:c r="A96" t="inlineStr">
@@ -4391,6 +5267,14 @@
       <x:c r="J96" t="n">
         <x:v>85</x:v>
       </x:c>
+      <x:c r="K96" t="str"/>
+      <x:c r="L96" t="str"/>
+      <x:c r="M96" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N96" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" t="inlineStr">
@@ -4433,6 +5317,14 @@
       <x:c r="J97" t="n">
         <x:v>85</x:v>
       </x:c>
+      <x:c r="K97" t="str"/>
+      <x:c r="L97" t="str"/>
+      <x:c r="M97" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N97" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="inlineStr">
@@ -4475,6 +5367,14 @@
       <x:c r="J98" t="n">
         <x:v>85</x:v>
       </x:c>
+      <x:c r="K98" t="str"/>
+      <x:c r="L98" t="str"/>
+      <x:c r="M98" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N98" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="99">
       <x:c r="A99" t="inlineStr">
@@ -4517,6 +5417,14 @@
       <x:c r="J99" t="n">
         <x:v>85</x:v>
       </x:c>
+      <x:c r="K99" t="str"/>
+      <x:c r="L99" t="str"/>
+      <x:c r="M99" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N99" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" t="inlineStr">
@@ -4559,6 +5467,14 @@
       <x:c r="J100" t="n">
         <x:v>150</x:v>
       </x:c>
+      <x:c r="K100" t="str"/>
+      <x:c r="L100" t="str"/>
+      <x:c r="M100" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N100" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" t="inlineStr">
@@ -4601,6 +5517,14 @@
       <x:c r="J101" t="n">
         <x:v>150</x:v>
       </x:c>
+      <x:c r="K101" t="str"/>
+      <x:c r="L101" t="str"/>
+      <x:c r="M101" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N101" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" t="inlineStr">
@@ -4643,6 +5567,14 @@
       <x:c r="J102" t="n">
         <x:v>150</x:v>
       </x:c>
+      <x:c r="K102" t="str"/>
+      <x:c r="L102" t="str"/>
+      <x:c r="M102" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N102" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="103">
       <x:c r="A103" t="inlineStr">
@@ -4685,6 +5617,14 @@
       <x:c r="J103" t="n">
         <x:v>150</x:v>
       </x:c>
+      <x:c r="K103" t="str"/>
+      <x:c r="L103" t="str"/>
+      <x:c r="M103" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N103" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="104">
       <x:c r="A104" t="inlineStr">
@@ -4727,6 +5667,14 @@
       <x:c r="J104" t="n">
         <x:v>150</x:v>
       </x:c>
+      <x:c r="K104" t="str"/>
+      <x:c r="L104" t="str"/>
+      <x:c r="M104" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N104" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" t="inlineStr">
@@ -4769,6 +5717,14 @@
       <x:c r="J105" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K105" t="str"/>
+      <x:c r="L105" t="str"/>
+      <x:c r="M105" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N105" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="106">
       <x:c r="A106" t="inlineStr">
@@ -4811,6 +5767,14 @@
       <x:c r="J106" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K106" t="str"/>
+      <x:c r="L106" t="str"/>
+      <x:c r="M106" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N106" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="107">
       <x:c r="A107" t="inlineStr">
@@ -4853,6 +5817,14 @@
       <x:c r="J107" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K107" t="str"/>
+      <x:c r="L107" t="str"/>
+      <x:c r="M107" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N107" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="108">
       <x:c r="A108" t="inlineStr">
@@ -4895,6 +5867,14 @@
       <x:c r="J108" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K108" t="str"/>
+      <x:c r="L108" t="str"/>
+      <x:c r="M108" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N108" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="109">
       <x:c r="A109" t="inlineStr">
@@ -4937,6 +5917,14 @@
       <x:c r="J109" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K109" t="str"/>
+      <x:c r="L109" t="str"/>
+      <x:c r="M109" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N109" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="A110" t="inlineStr">
@@ -4979,6 +5967,14 @@
       <x:c r="J110" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K110" t="str"/>
+      <x:c r="L110" t="str"/>
+      <x:c r="M110" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N110" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="111">
       <x:c r="A111" t="inlineStr">
@@ -5021,6 +6017,14 @@
       <x:c r="J111" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K111" t="str"/>
+      <x:c r="L111" t="str"/>
+      <x:c r="M111" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N111" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" t="inlineStr">
@@ -5063,6 +6067,14 @@
       <x:c r="J112" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K112" t="str"/>
+      <x:c r="L112" t="str"/>
+      <x:c r="M112" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N112" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" t="inlineStr">
@@ -5105,6 +6117,14 @@
       <x:c r="J113" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K113" t="str"/>
+      <x:c r="L113" t="str"/>
+      <x:c r="M113" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N113" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" t="inlineStr">
@@ -5147,6 +6167,14 @@
       <x:c r="J114" t="n">
         <x:v>90</x:v>
       </x:c>
+      <x:c r="K114" t="str"/>
+      <x:c r="L114" t="str"/>
+      <x:c r="M114" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N114" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" t="inlineStr">
@@ -5189,6 +6217,14 @@
       <x:c r="J115" t="n">
         <x:v>95</x:v>
       </x:c>
+      <x:c r="K115" t="str"/>
+      <x:c r="L115" t="str"/>
+      <x:c r="M115" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N115" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" t="inlineStr">
@@ -5231,6 +6267,14 @@
       <x:c r="J116" t="n">
         <x:v>95</x:v>
       </x:c>
+      <x:c r="K116" t="str"/>
+      <x:c r="L116" t="str"/>
+      <x:c r="M116" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N116" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" t="inlineStr">
@@ -5273,6 +6317,14 @@
       <x:c r="J117" t="n">
         <x:v>95</x:v>
       </x:c>
+      <x:c r="K117" t="str"/>
+      <x:c r="L117" t="str"/>
+      <x:c r="M117" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N117" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" t="inlineStr">
@@ -5315,6 +6367,14 @@
       <x:c r="J118" t="n">
         <x:v>95</x:v>
       </x:c>
+      <x:c r="K118" t="str"/>
+      <x:c r="L118" t="str"/>
+      <x:c r="M118" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N118" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" t="inlineStr">
@@ -5357,6 +6417,14 @@
       <x:c r="J119" t="n">
         <x:v>95</x:v>
       </x:c>
+      <x:c r="K119" t="str"/>
+      <x:c r="L119" t="str"/>
+      <x:c r="M119" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N119" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" t="inlineStr">
@@ -5399,6 +6467,14 @@
       <x:c r="J120" t="n">
         <x:v>95</x:v>
       </x:c>
+      <x:c r="K120" t="str"/>
+      <x:c r="L120" t="str"/>
+      <x:c r="M120" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N120" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="121">
       <x:c r="A121" t="inlineStr">
@@ -5441,6 +6517,14 @@
       <x:c r="J121" t="n">
         <x:v>95</x:v>
       </x:c>
+      <x:c r="K121" t="str"/>
+      <x:c r="L121" t="str"/>
+      <x:c r="M121" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N121" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" t="inlineStr">
@@ -5483,6 +6567,14 @@
       <x:c r="J122" t="n">
         <x:v>95</x:v>
       </x:c>
+      <x:c r="K122" t="str"/>
+      <x:c r="L122" t="str"/>
+      <x:c r="M122" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N122" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" t="inlineStr">
@@ -5525,6 +6617,14 @@
       <x:c r="J123" t="n">
         <x:v>95</x:v>
       </x:c>
+      <x:c r="K123" t="str"/>
+      <x:c r="L123" t="str"/>
+      <x:c r="M123" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N123" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" t="inlineStr">
@@ -5567,6 +6667,14 @@
       <x:c r="J124" t="n">
         <x:v>145</x:v>
       </x:c>
+      <x:c r="K124" t="str"/>
+      <x:c r="L124" t="str"/>
+      <x:c r="M124" s="2" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="N124" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" t="inlineStr">
@@ -5609,6 +6717,14 @@
       <x:c r="J125" t="n">
         <x:v>145</x:v>
       </x:c>
+      <x:c r="K125" t="str"/>
+      <x:c r="L125" t="str"/>
+      <x:c r="M125" s="2" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="N125" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" t="inlineStr">
@@ -5651,6 +6767,14 @@
       <x:c r="J126" t="n">
         <x:v>145</x:v>
       </x:c>
+      <x:c r="K126" t="str"/>
+      <x:c r="L126" t="str"/>
+      <x:c r="M126" s="2" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="N126" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" t="inlineStr">
@@ -5693,6 +6817,14 @@
       <x:c r="J127" t="n">
         <x:v>145</x:v>
       </x:c>
+      <x:c r="K127" t="str"/>
+      <x:c r="L127" t="str"/>
+      <x:c r="M127" s="2" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="N127" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" t="inlineStr">
@@ -5735,6 +6867,14 @@
       <x:c r="J128" t="n">
         <x:v>145</x:v>
       </x:c>
+      <x:c r="K128" t="str"/>
+      <x:c r="L128" t="str"/>
+      <x:c r="M128" s="2" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="N128" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="A129" t="inlineStr">
@@ -5777,6 +6917,14 @@
       <x:c r="J129" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K129" t="str"/>
+      <x:c r="L129" t="str"/>
+      <x:c r="M129" s="2" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="N129" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" t="inlineStr">
@@ -5819,6 +6967,14 @@
       <x:c r="J130" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K130" t="str"/>
+      <x:c r="L130" t="str"/>
+      <x:c r="M130" s="2" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="N130" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" t="inlineStr">
@@ -5861,6 +7017,14 @@
       <x:c r="J131" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K131" t="str"/>
+      <x:c r="L131" t="str"/>
+      <x:c r="M131" s="2" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="N131" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" t="inlineStr">
@@ -5903,6 +7067,14 @@
       <x:c r="J132" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K132" t="str"/>
+      <x:c r="L132" t="str"/>
+      <x:c r="M132" s="2" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="N132" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" t="inlineStr">
@@ -5945,6 +7117,14 @@
       <x:c r="J133" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K133" t="str"/>
+      <x:c r="L133" t="str"/>
+      <x:c r="M133" s="2" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="N133" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" t="inlineStr">
@@ -5987,6 +7167,14 @@
       <x:c r="J134" t="n">
         <x:v>155</x:v>
       </x:c>
+      <x:c r="K134" t="str"/>
+      <x:c r="L134" t="str"/>
+      <x:c r="M134" s="2" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="N134" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" t="inlineStr">
@@ -6029,6 +7217,14 @@
       <x:c r="J135" t="n">
         <x:v>185</x:v>
       </x:c>
+      <x:c r="K135" t="str"/>
+      <x:c r="L135" t="str"/>
+      <x:c r="M135" s="2" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="N135" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" t="inlineStr">
@@ -6071,6 +7267,14 @@
       <x:c r="J136" t="n">
         <x:v>75</x:v>
       </x:c>
+      <x:c r="K136" t="str"/>
+      <x:c r="L136" t="str"/>
+      <x:c r="M136" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="N136" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" t="inlineStr">
@@ -6113,6 +7317,14 @@
       <x:c r="J137" t="n">
         <x:v>125</x:v>
       </x:c>
+      <x:c r="K137" t="str"/>
+      <x:c r="L137" t="str"/>
+      <x:c r="M137" s="2" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="N137" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" t="inlineStr">
@@ -6155,6 +7367,14 @@
       <x:c r="J138" t="n">
         <x:v>170</x:v>
       </x:c>
+      <x:c r="K138" t="str"/>
+      <x:c r="L138" t="str"/>
+      <x:c r="M138" s="2" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="N138" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" t="inlineStr">
@@ -6197,6 +7417,14 @@
       <x:c r="J139" t="n">
         <x:v>60</x:v>
       </x:c>
+      <x:c r="K139" t="str"/>
+      <x:c r="L139" t="str"/>
+      <x:c r="M139" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N139" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="140">
       <x:c r="A140" t="inlineStr">
@@ -6239,6 +7467,14 @@
       <x:c r="J140" t="n">
         <x:v>75</x:v>
       </x:c>
+      <x:c r="K140" t="str"/>
+      <x:c r="L140" t="str"/>
+      <x:c r="M140" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N140" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="141">
       <x:c r="A141" t="inlineStr">
@@ -6281,6 +7517,14 @@
       <x:c r="J141" t="n">
         <x:v>120</x:v>
       </x:c>
+      <x:c r="K141" t="str"/>
+      <x:c r="L141" t="str"/>
+      <x:c r="M141" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="N141" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" t="inlineStr">
@@ -6323,6 +7567,14 @@
       <x:c r="J142" t="n">
         <x:v>115</x:v>
       </x:c>
+      <x:c r="K142" t="str"/>
+      <x:c r="L142" t="str"/>
+      <x:c r="M142" s="2" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="N142" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="143">
       <x:c r="A143" t="inlineStr">
@@ -6365,6 +7617,14 @@
       <x:c r="J143" t="n">
         <x:v>215</x:v>
       </x:c>
+      <x:c r="K143" t="str"/>
+      <x:c r="L143" t="str"/>
+      <x:c r="M143" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N143" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="144">
       <x:c r="A144" t="inlineStr">
@@ -6407,6 +7667,14 @@
       <x:c r="J144" t="n">
         <x:v>135</x:v>
       </x:c>
+      <x:c r="K144" t="str"/>
+      <x:c r="L144" t="str"/>
+      <x:c r="M144" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="N144" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="145">
       <x:c r="A145" t="inlineStr">
@@ -6449,6 +7717,14 @@
       <x:c r="J145" t="n">
         <x:v>100</x:v>
       </x:c>
+      <x:c r="K145" t="str"/>
+      <x:c r="L145" t="str"/>
+      <x:c r="M145" s="2" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N145" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="146">
       <x:c r="A146" t="inlineStr">
@@ -6490,6 +7766,454 @@
       </x:c>
       <x:c r="J146" t="n">
         <x:v>100</x:v>
+      </x:c>
+      <x:c r="K146" t="str"/>
+      <x:c r="L146" t="str"/>
+      <x:c r="M146" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="N146" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" t="str">
+        <x:v>cabinet_01</x:v>
+      </x:c>
+      <x:c r="B147" t="str">
+        <x:v>cabinet_01</x:v>
+      </x:c>
+      <x:c r="C147" t="str">
+        <x:v>立柜·01</x:v>
+      </x:c>
+      <x:c r="D147" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="E147" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="F147" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G147" t="str">
+        <x:v>Assets/PC ui/Scene/furniture/cabinet_01.png</x:v>
+      </x:c>
+      <x:c r="H147" t="str">
+        <x:v>#DBC4A0</x:v>
+      </x:c>
+      <x:c r="I147" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="J147" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="K147" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/Frame 114.png</x:v>
+      </x:c>
+      <x:c r="L147" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/Frame 104.png</x:v>
+      </x:c>
+      <x:c r="M147" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N147" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" t="str">
+        <x:v>cabinet_02</x:v>
+      </x:c>
+      <x:c r="B148" t="str">
+        <x:v>cabinet_02</x:v>
+      </x:c>
+      <x:c r="C148" t="str">
+        <x:v>立柜·02</x:v>
+      </x:c>
+      <x:c r="D148" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="E148" t="n">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="F148" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G148" t="str">
+        <x:v>Assets/PC ui/Scene/furniture/cabinet_02.png</x:v>
+      </x:c>
+      <x:c r="H148" t="str">
+        <x:v>#E8B2A6</x:v>
+      </x:c>
+      <x:c r="I148" t="n">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="J148" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="K148" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/Frame 115.png</x:v>
+      </x:c>
+      <x:c r="L148" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/Frame 105.png</x:v>
+      </x:c>
+      <x:c r="M148" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N148" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" t="str">
+        <x:v>cabinet_03</x:v>
+      </x:c>
+      <x:c r="B149" t="str">
+        <x:v>cabinet_03</x:v>
+      </x:c>
+      <x:c r="C149" t="str">
+        <x:v>立柜·03</x:v>
+      </x:c>
+      <x:c r="D149" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="E149" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="F149" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G149" t="str">
+        <x:v>Assets/PC ui/Scene/furniture/cabinet_03.png</x:v>
+      </x:c>
+      <x:c r="H149" t="str">
+        <x:v>#959E78</x:v>
+      </x:c>
+      <x:c r="I149" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="J149" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="K149" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/Frame 113.png</x:v>
+      </x:c>
+      <x:c r="L149" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/Frame 103.png</x:v>
+      </x:c>
+      <x:c r="M149" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="N149" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" t="str">
+        <x:v>cabinet_04</x:v>
+      </x:c>
+      <x:c r="B150" t="str">
+        <x:v>cabinet_04</x:v>
+      </x:c>
+      <x:c r="C150" t="str">
+        <x:v>立柜·04</x:v>
+      </x:c>
+      <x:c r="D150" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="E150" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="F150" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G150" t="str">
+        <x:v>Assets/PC ui/Scene/furniture/cabinet_04.png</x:v>
+      </x:c>
+      <x:c r="H150" t="str">
+        <x:v>#ADC2C8</x:v>
+      </x:c>
+      <x:c r="I150" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="J150" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="K150" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/Frame 112.png</x:v>
+      </x:c>
+      <x:c r="L150" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/Frame 102.png</x:v>
+      </x:c>
+      <x:c r="M150" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N150" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" t="str">
+        <x:v>cabinet_05</x:v>
+      </x:c>
+      <x:c r="B151" t="str">
+        <x:v>cabinet_05</x:v>
+      </x:c>
+      <x:c r="C151" t="str">
+        <x:v>立柜·05</x:v>
+      </x:c>
+      <x:c r="D151" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="E151" t="n">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="F151" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G151" t="str">
+        <x:v>Assets/PC ui/Scene/furniture/cabinet_05.png</x:v>
+      </x:c>
+      <x:c r="H151" t="str">
+        <x:v>#BFAEC4</x:v>
+      </x:c>
+      <x:c r="I151" t="n">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="J151" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="K151" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/Frame 111.png</x:v>
+      </x:c>
+      <x:c r="L151" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/Frame 101.png</x:v>
+      </x:c>
+      <x:c r="M151" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N151" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" t="str">
+        <x:v>cabinet_06</x:v>
+      </x:c>
+      <x:c r="B152" t="str">
+        <x:v>cabinet_06</x:v>
+      </x:c>
+      <x:c r="C152" t="str">
+        <x:v>立柜·06</x:v>
+      </x:c>
+      <x:c r="D152" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="E152" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="F152" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G152" t="str">
+        <x:v>Assets/PC ui/Scene/furniture/cabinet_06.png</x:v>
+      </x:c>
+      <x:c r="H152" t="str">
+        <x:v>#D9A566</x:v>
+      </x:c>
+      <x:c r="I152" t="n">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="J152" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="K152" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/Frame 110.png</x:v>
+      </x:c>
+      <x:c r="L152" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/Frame 100.png</x:v>
+      </x:c>
+      <x:c r="M152" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N152" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" t="str">
+        <x:v>cabinet_07</x:v>
+      </x:c>
+      <x:c r="B153" t="str">
+        <x:v>cabinet_07</x:v>
+      </x:c>
+      <x:c r="C153" t="str">
+        <x:v>立柜·07</x:v>
+      </x:c>
+      <x:c r="D153" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="E153" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="F153" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G153" t="str">
+        <x:v>Assets/PC ui/Scene/furniture/cabinet_07.png</x:v>
+      </x:c>
+      <x:c r="H153" t="str">
+        <x:v>#ABBBBF</x:v>
+      </x:c>
+      <x:c r="I153" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="J153" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="K153" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/Frame 109.png</x:v>
+      </x:c>
+      <x:c r="L153" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/Frame 99.png</x:v>
+      </x:c>
+      <x:c r="M153" s="2" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="N153" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" t="str">
+        <x:v>cabinet_08</x:v>
+      </x:c>
+      <x:c r="B154" t="str">
+        <x:v>cabinet_08</x:v>
+      </x:c>
+      <x:c r="C154" t="str">
+        <x:v>立柜·08</x:v>
+      </x:c>
+      <x:c r="D154" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="E154" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="F154" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G154" t="str">
+        <x:v>Assets/PC ui/Scene/furniture/cabinet_08.png</x:v>
+      </x:c>
+      <x:c r="H154" t="str">
+        <x:v>#BEB0A0</x:v>
+      </x:c>
+      <x:c r="I154" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="J154" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="K154" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/Frame 116.png</x:v>
+      </x:c>
+      <x:c r="L154" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/Frame 106.png</x:v>
+      </x:c>
+      <x:c r="M154" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N154" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" t="str">
+        <x:v>cabinet_09</x:v>
+      </x:c>
+      <x:c r="B155" t="str">
+        <x:v>cabinet_09</x:v>
+      </x:c>
+      <x:c r="C155" t="str">
+        <x:v>立柜·09</x:v>
+      </x:c>
+      <x:c r="D155" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="E155" t="n">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="F155" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G155" t="str">
+        <x:v>Assets/PC ui/Scene/furniture/cabinet_09.png</x:v>
+      </x:c>
+      <x:c r="H155" t="str">
+        <x:v>#E59179</x:v>
+      </x:c>
+      <x:c r="I155" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="J155" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="K155" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/Frame 117.png</x:v>
+      </x:c>
+      <x:c r="L155" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/Frame 107.png</x:v>
+      </x:c>
+      <x:c r="M155" s="2" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="N155" s="2" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" t="str">
+        <x:v>cabinet_10</x:v>
+      </x:c>
+      <x:c r="B156" t="str">
+        <x:v>cabinet_10</x:v>
+      </x:c>
+      <x:c r="C156" t="str">
+        <x:v>立柜·10</x:v>
+      </x:c>
+      <x:c r="D156" t="str">
+        <x:v>cabinet</x:v>
+      </x:c>
+      <x:c r="E156" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="F156" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="G156" t="str">
+        <x:v>Assets/PC ui/Scene/furniture/cabinet_10.png</x:v>
+      </x:c>
+      <x:c r="H156" t="str">
+        <x:v>#AAC1BF</x:v>
+      </x:c>
+      <x:c r="I156" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="J156" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="K156" t="str">
+        <x:v>Assets/PC ui 2.0/store/左侧家具图标/Frame 108.png</x:v>
+      </x:c>
+      <x:c r="L156" t="str">
+        <x:v>Assets/PC ui 2.0/store/右侧家具图标/Frame 98.png</x:v>
+      </x:c>
+      <x:c r="M156" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N156" s="2" t="n">
+        <x:v>7</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>